<commit_message>
fix: remove Package Types tab, fix 84 off-by-one VLOOKUP formulas in Package Selector, remove Guest Package margin row
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Packages_12Variations.xlsx
+++ b/files/LA_Golf_Packages_12Variations.xlsx
@@ -7,10 +7,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Types" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guest Package" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guest Package" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -3002,513 +3001,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FFD4AF37"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" style="42" min="1" max="1"/>
-    <col width="3.7109375" bestFit="1" customWidth="1" style="42" min="2" max="2"/>
-    <col width="5.7109375" bestFit="1" customWidth="1" style="42" min="3" max="3"/>
-    <col width="12" customWidth="1" style="42" min="4" max="4"/>
-    <col width="3" bestFit="1" customWidth="1" style="42" min="5" max="6"/>
-    <col width="4" bestFit="1" customWidth="1" style="42" min="7" max="7"/>
-    <col width="14" customWidth="1" style="42" min="8" max="8"/>
-    <col width="6.28515625" bestFit="1" customWidth="1" style="42" min="9" max="9"/>
-    <col width="6.140625" bestFit="1" customWidth="1" style="42" min="10" max="10"/>
-    <col width="6.28515625" bestFit="1" customWidth="1" style="42" min="11" max="11"/>
-    <col width="6.140625" bestFit="1" customWidth="1" style="42" min="12" max="12"/>
-    <col width="5.140625" bestFit="1" customWidth="1" style="42" min="13" max="13"/>
-    <col width="7.28515625" bestFit="1" customWidth="1" style="42" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="38.25" customHeight="1" s="42">
-      <c r="A1" s="32" t="inlineStr">
-        <is>
-          <t>🎯 결 TOUR — 대표 패키지 (1인 기준, USD | 중복코스 없음)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="37" t="inlineStr">
-        <is>
-          <t>⚠️ 참고용 대표패키지 → 'Package Selector' 시트에서 자유롭게 커스터마이징</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16.5" customHeight="1" s="42">
-      <c r="A4" s="76" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B4" s="76" t="inlineStr">
-        <is>
-          <t>일정</t>
-        </is>
-      </c>
-      <c r="C4" s="76" t="inlineStr">
-        <is>
-          <t>패키지명</t>
-        </is>
-      </c>
-      <c r="D4" s="76" t="inlineStr">
-        <is>
-          <t>박</t>
-        </is>
-      </c>
-      <c r="E4" s="76" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="F4" s="76" t="inlineStr">
-        <is>
-          <t>Rds</t>
-        </is>
-      </c>
-      <c r="G4" s="76" t="inlineStr">
-        <is>
-          <t>패키지 구성</t>
-        </is>
-      </c>
-      <c r="H4" s="77" t="inlineStr">
-        <is>
-          <t>⛳ 골프</t>
-        </is>
-      </c>
-      <c r="I4" s="150" t="n"/>
-      <c r="J4" s="150" t="n"/>
-      <c r="K4" s="150" t="n"/>
-      <c r="L4" s="150" t="n"/>
-      <c r="M4" s="150" t="n"/>
-      <c r="N4" s="150" t="n"/>
-      <c r="O4" s="92" t="n"/>
-      <c r="P4" s="77" t="inlineStr">
-        <is>
-          <t>🍽️ 식사</t>
-        </is>
-      </c>
-      <c r="Q4" s="92" t="n"/>
-      <c r="R4" s="77" t="inlineStr">
-        <is>
-          <t>📦 기타</t>
-        </is>
-      </c>
-      <c r="S4" s="92" t="n"/>
-      <c r="T4" s="76" t="inlineStr">
-        <is>
-          <t>마진</t>
-        </is>
-      </c>
-      <c r="U4" s="76" t="inlineStr">
-        <is>
-          <t>마진율</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="51" customHeight="1" s="42">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="78" t="n"/>
-      <c r="C5" s="78" t="n"/>
-      <c r="D5" s="78" t="n"/>
-      <c r="E5" s="78" t="n"/>
-      <c r="F5" s="78" t="n"/>
-      <c r="G5" s="78" t="n"/>
-      <c r="H5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="I5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="J5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="K5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="L5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="M5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="N5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="O5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="P5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="Q5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="R5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="S5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="T5" s="148" t="inlineStr"/>
-      <c r="U5" s="148" t="inlineStr"/>
-    </row>
-    <row r="6" ht="51" customHeight="1" s="42">
-      <c r="A6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>트럼프 + 샌드파이퍼 오션뷰</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Trump×1 + Sand×1</t>
-        </is>
-      </c>
-      <c r="H6" s="149" t="inlineStr">
-        <is>
-          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>745</v>
-      </c>
-      <c r="J6" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="79" t="n">
-        <v>120</v>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N6" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="O6" s="79" t="n">
-        <v>525</v>
-      </c>
-      <c r="P6" s="79" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q6" s="79" t="n">
-        <v>1215</v>
-      </c>
-      <c r="R6" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="S6" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="T6" s="79">
-        <f>(J6+L6+N6+P6+R6+T6)-(I6+K6+M6+O6+Q6+S6)</f>
-        <v/>
-      </c>
-      <c r="U6" s="80">
-        <f>IF(J6+L6+N6+P6+R6+T6&gt;0,((J6+L6+N6+P6+R6+T6)-(I6+K6+M6+O6+Q6+S6))/(J6+L6+N6+P6+R6+T6),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="34.5" customHeight="1" s="42">
-      <c r="A7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>트럼프 + 히든밸리 밸리뷰</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Trump×1 + HV×1</t>
-        </is>
-      </c>
-      <c r="H7" s="149" t="inlineStr">
-        <is>
-          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>609</v>
-      </c>
-      <c r="J7" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="K7" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="L7" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N7" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="O7" s="79" t="n">
-        <v>525</v>
-      </c>
-      <c r="P7" s="79" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q7" s="79" t="n">
-        <v>1215</v>
-      </c>
-      <c r="R7" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="S7" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="T7" s="79">
-        <f>(J7+L7+N7+P7+R7+T7)-(I7+K7+M7+O7+Q7+S7)</f>
-        <v/>
-      </c>
-      <c r="U7" s="80">
-        <f>IF(J7+L7+N7+P7+R7+T7&gt;0,((J7+L7+N7+P7+R7+T7)-(I7+K7+M7+O7+Q7+S7))/(J7+L7+N7+P7+R7+T7),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>샌드파이퍼 + 히든밸리</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Sand×1 + HV×1</t>
-        </is>
-      </c>
-      <c r="H8" s="149" t="inlineStr">
-        <is>
-          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>354</v>
-      </c>
-      <c r="J8" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="K8" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N8" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="O8" s="79" t="n">
-        <v>525</v>
-      </c>
-      <c r="P8" s="79" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q8" s="79" t="n">
-        <v>1215</v>
-      </c>
-      <c r="R8" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="S8" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="T8" s="79">
-        <f>(J8+L8+N8+P8+R8+T8)-(I8+K8+M8+O8+Q8+S8)</f>
-        <v/>
-      </c>
-      <c r="U8" s="80">
-        <f>IF(J8+L8+N8+P8+R8+T8&gt;0,((J8+L8+N8+P8+R8+T8)-(I8+K8+M8+O8+Q8+S8))/(J8+L8+N8+P8+R8+T8),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="51" customHeight="1" s="42">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n"/>
-      <c r="L9" s="10" t="n"/>
-      <c r="M9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>5N7D</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>트럼프+샌드+히든 3色 시그니처</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Trump×1+Sand×1+HV×1</t>
-        </is>
-      </c>
-      <c r="H10" s="149" t="inlineStr">
-        <is>
-          <t>G3·H5·T5·M5B5L5D2Ex·I5</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>854</v>
-      </c>
-      <c r="J10" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="K10" s="79" t="n">
-        <v>165</v>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>1375</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>1875</v>
-      </c>
-      <c r="N10" s="79" t="n">
-        <v>625</v>
-      </c>
-      <c r="O10" s="79" t="n">
-        <v>875</v>
-      </c>
-      <c r="P10" s="79" t="n">
-        <v>1350</v>
-      </c>
-      <c r="Q10" s="79" t="n">
-        <v>2025</v>
-      </c>
-      <c r="R10" s="79" t="n">
-        <v>250</v>
-      </c>
-      <c r="S10" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="T10" s="79">
-        <f>(J10+L10+N10+P10+R10+T10)-(I10+K10+M10+O10+Q10+S10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="80">
-        <f>IF(J10+L10+N10+P10+R10+T10&gt;0,((J10+L10+N10+P10+R10+T10)-(I10+K10+M10+O10+Q10+S10))/(J10+L10+N10+P10+R10+T10),0)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="R4:S4"/>
-    <mergeCell ref="H4:O4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3806,15 +3298,15 @@
         <v>1</v>
       </c>
       <c r="C11" s="84">
-        <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D11" s="84">
-        <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E11" s="137">
-        <f>IF(D10&gt;0,(D10-C10)/D10,0)</f>
+        <f>IF(D11&gt;0,(D11-C11)/D11,0)</f>
         <v/>
       </c>
       <c r="F11" s="145" t="inlineStr"/>
@@ -3848,15 +3340,15 @@
         <v>2</v>
       </c>
       <c r="C12" s="84">
-        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D12" s="84">
-        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E12" s="137">
-        <f>IF(D11&gt;0,(D11-C11)/D11,0)</f>
+        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
         <v/>
       </c>
       <c r="F12" s="145" t="inlineStr"/>
@@ -3890,15 +3382,15 @@
         <v>2</v>
       </c>
       <c r="C13" s="84">
-        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D13" s="84">
-        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E13" s="137">
-        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
+        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
         <v/>
       </c>
       <c r="F13" s="145" t="inlineStr"/>
@@ -3926,15 +3418,15 @@
       <c r="A14" s="129" t="inlineStr"/>
       <c r="B14" s="83" t="inlineStr"/>
       <c r="C14" s="84">
-        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D14" s="84">
-        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E14" s="137">
-        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
+        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
         <v/>
       </c>
       <c r="F14" s="145" t="inlineStr"/>
@@ -3962,15 +3454,15 @@
       <c r="A15" s="129" t="inlineStr"/>
       <c r="B15" s="83" t="inlineStr"/>
       <c r="C15" s="84">
-        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D15" s="84">
-        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E15" s="137">
-        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
+        <f>IF(D15&gt;0,(D15-C15)/D15,0)</f>
         <v/>
       </c>
       <c r="F15" s="145" t="inlineStr"/>
@@ -4078,15 +3570,15 @@
         <v>3</v>
       </c>
       <c r="C19" s="84">
-        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D19" s="84">
-        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E19" s="137">
-        <f>IF(D18&gt;0,(D18-C18)/D18,0)</f>
+        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
         <v/>
       </c>
       <c r="F19" s="145" t="inlineStr"/>
@@ -4114,15 +3606,15 @@
       <c r="A20" s="129" t="inlineStr"/>
       <c r="B20" s="83" t="inlineStr"/>
       <c r="C20" s="84">
-        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D20" s="84">
-        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E20" s="137">
-        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
+        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
         <v/>
       </c>
       <c r="F20" s="145" t="inlineStr"/>
@@ -4150,15 +3642,15 @@
       <c r="A21" s="129" t="inlineStr"/>
       <c r="B21" s="83" t="inlineStr"/>
       <c r="C21" s="84">
-        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A21="","",VLOOKUP(A21,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D21" s="84">
-        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A21="","",VLOOKUP(A21,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E21" s="137">
-        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
+        <f>IF(D21&gt;0,(D21-C21)/D21,0)</f>
         <v/>
       </c>
       <c r="F21" s="145" t="inlineStr"/>
@@ -4266,15 +3758,15 @@
         <v>3</v>
       </c>
       <c r="C25" s="84">
-        <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D25" s="84">
-        <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E25" s="137">
-        <f>IF(D24&gt;0,(D24-C24)/D24,0)</f>
+        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
         <v/>
       </c>
       <c r="F25" s="145" t="inlineStr"/>
@@ -4302,15 +3794,15 @@
       <c r="A26" s="129" t="inlineStr"/>
       <c r="B26" s="83" t="inlineStr"/>
       <c r="C26" s="84">
-        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D26" s="84">
-        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E26" s="137">
-        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
+        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
         <v/>
       </c>
       <c r="F26" s="145" t="inlineStr"/>
@@ -4338,15 +3830,15 @@
       <c r="A27" s="129" t="inlineStr"/>
       <c r="B27" s="83" t="inlineStr"/>
       <c r="C27" s="84">
-        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D27" s="84">
-        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E27" s="137">
-        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
+        <f>IF(D27&gt;0,(D27-C27)/D27,0)</f>
         <v/>
       </c>
       <c r="F27" s="145" t="inlineStr"/>
@@ -4454,15 +3946,15 @@
         <v>3</v>
       </c>
       <c r="C31" s="84">
-        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D31" s="84">
-        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E31" s="137">
-        <f>IF(D30&gt;0,(D30-C30)/D30,0)</f>
+        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
         <v/>
       </c>
       <c r="F31" s="145" t="inlineStr"/>
@@ -4496,15 +3988,15 @@
         <v>3</v>
       </c>
       <c r="C32" s="84">
-        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D32" s="84">
-        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E32" s="137">
-        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
+        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
         <v/>
       </c>
       <c r="F32" s="145" t="inlineStr"/>
@@ -4538,15 +4030,15 @@
         <v>2</v>
       </c>
       <c r="C33" s="84">
-        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D33" s="84">
-        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E33" s="137">
-        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
+        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
         <v/>
       </c>
       <c r="F33" s="145" t="inlineStr"/>
@@ -4580,15 +4072,15 @@
         <v>3</v>
       </c>
       <c r="C34" s="84">
-        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D34" s="84">
-        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E34" s="137">
-        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
+        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
         <v/>
       </c>
       <c r="F34" s="145" t="inlineStr"/>
@@ -4616,15 +4108,15 @@
       <c r="A35" s="129" t="inlineStr"/>
       <c r="B35" s="83" t="inlineStr"/>
       <c r="C35" s="84">
-        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D35" s="84">
-        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E35" s="137">
-        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
+        <f>IF(D35&gt;0,(D35-C35)/D35,0)</f>
         <v/>
       </c>
       <c r="F35" s="145" t="inlineStr"/>
@@ -4732,15 +4224,15 @@
         <v>4</v>
       </c>
       <c r="C39" s="84">
-        <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D39" s="84">
-        <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E39" s="137">
-        <f>IF(D38&gt;0,(D38-C38)/D38,0)</f>
+        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
         <v/>
       </c>
       <c r="F39" s="145" t="inlineStr"/>
@@ -4768,15 +4260,15 @@
       <c r="A40" s="129" t="inlineStr"/>
       <c r="B40" s="83" t="inlineStr"/>
       <c r="C40" s="84">
-        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D40" s="84">
-        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E40" s="137">
-        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
+        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
         <v/>
       </c>
       <c r="F40" s="145" t="inlineStr"/>
@@ -4804,15 +4296,15 @@
       <c r="A41" s="129" t="inlineStr"/>
       <c r="B41" s="83" t="inlineStr"/>
       <c r="C41" s="84">
-        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D41" s="84">
-        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E41" s="137">
-        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
+        <f>IF(D41&gt;0,(D41-C41)/D41,0)</f>
         <v/>
       </c>
       <c r="F41" s="145" t="inlineStr"/>
@@ -4920,15 +4412,15 @@
         <v>1</v>
       </c>
       <c r="C45" s="84">
-        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D45" s="84">
-        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E45" s="137">
-        <f>IF(D44&gt;0,(D44-C44)/D44,0)</f>
+        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
         <v/>
       </c>
       <c r="F45" s="145" t="inlineStr"/>
@@ -4962,15 +4454,15 @@
         <v>1</v>
       </c>
       <c r="C46" s="84">
-        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D46" s="84">
-        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E46" s="137">
-        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
+        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
         <v/>
       </c>
       <c r="F46" s="145" t="inlineStr"/>
@@ -5004,15 +4496,15 @@
         <v>1</v>
       </c>
       <c r="C47" s="84">
-        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D47" s="84">
-        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E47" s="137">
-        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
+        <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
         <v/>
       </c>
       <c r="F47" s="145" t="inlineStr"/>
@@ -5046,15 +4538,15 @@
         <v>1</v>
       </c>
       <c r="C48" s="84">
-        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D48" s="84">
-        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E48" s="137">
-        <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
+        <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
         <v/>
       </c>
       <c r="F48" s="145" t="inlineStr"/>
@@ -5082,15 +4574,15 @@
       <c r="A49" s="129" t="inlineStr"/>
       <c r="B49" s="83" t="inlineStr"/>
       <c r="C49" s="84">
-        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D49" s="84">
-        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E49" s="137">
-        <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
+        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
         <v/>
       </c>
       <c r="F49" s="145" t="inlineStr"/>
@@ -5118,15 +4610,15 @@
       <c r="A50" s="129" t="inlineStr"/>
       <c r="B50" s="83" t="inlineStr"/>
       <c r="C50" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D50" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E50" s="137">
-        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
+        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
         <v/>
       </c>
       <c r="F50" s="145" t="inlineStr"/>
@@ -5154,15 +4646,15 @@
       <c r="A51" s="129" t="inlineStr"/>
       <c r="B51" s="83" t="inlineStr"/>
       <c r="C51" s="84">
-        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D51" s="84">
-        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E51" s="137">
-        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
+        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
         <v/>
       </c>
       <c r="F51" s="145" t="inlineStr"/>
@@ -5190,15 +4682,15 @@
       <c r="A52" s="129" t="inlineStr"/>
       <c r="B52" s="83" t="inlineStr"/>
       <c r="C52" s="84">
-        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D52" s="84">
-        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E52" s="137">
-        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
+        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
         <v/>
       </c>
       <c r="F52" s="145" t="inlineStr"/>
@@ -5226,15 +4718,15 @@
       <c r="A53" s="129" t="inlineStr"/>
       <c r="B53" s="83" t="inlineStr"/>
       <c r="C53" s="84">
-        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D53" s="84">
-        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E53" s="137">
-        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
+        <f>IF(D53&gt;0,(D53-C53)/D53,0)</f>
         <v/>
       </c>
       <c r="F53" s="145" t="inlineStr"/>
@@ -5309,6 +4801,7 @@
         <v/>
       </c>
     </row>
+    <row r="55"/>
     <row r="56"/>
     <row r="57">
       <c r="A57" s="103" t="inlineStr">
@@ -6406,7 +5899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6664,7 +6157,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6689,6 +6182,7 @@
       <c r="C1" s="150" t="n"/>
       <c r="D1" s="92" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="106" t="inlineStr">
         <is>
@@ -6731,6 +6225,7 @@
       <c r="C5" s="86" t="n"/>
       <c r="D5" s="87" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="124" t="inlineStr">
         <is>
@@ -6825,6 +6320,7 @@
       <c r="C13" s="86" t="n"/>
       <c r="D13" s="87" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="104" t="inlineStr"/>
       <c r="B15" s="150" t="n"/>
@@ -6861,25 +6357,11 @@
         </is>
       </c>
       <c r="B18" s="154">
-        <f>IF(B4&gt;0,B11/B4,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="106" t="inlineStr">
-        <is>
-          <t>Margin:</t>
-        </is>
-      </c>
-      <c r="B19" s="155">
-        <f>B11-B14</f>
-        <v/>
-      </c>
-      <c r="C19" s="156">
-        <f>IF(B11&gt;0,B13/B11,0)</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(B4&gt;0,B17/B4,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B10:D10"/>

</xml_diff>